<commit_message>
Formated main metrics and added addtional metrics.
</commit_message>
<xml_diff>
--- a/Word/rezultati.xlsx
+++ b/Word/rezultati.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\source\repos\omarkurtovic\ml-dotnet-vs-python\Word\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771DA4EC-51AB-4028-B9B9-4DEEA3E71D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F875A91-59F2-4F3D-9848-26D8574E0742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4EAF71C1-AA1B-4CDB-9B0B-819C93A82BA1}"/>
+    <workbookView xWindow="-28920" yWindow="5355" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4EAF71C1-AA1B-4CDB-9B0B-819C93A82BA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>C# 1</t>
   </si>
@@ -91,13 +92,52 @@
   </si>
   <si>
     <t>Prosjek  ± SD</t>
+  </si>
+  <si>
+    <t>Odziv N</t>
+  </si>
+  <si>
+    <t>F1 skor N</t>
+  </si>
+  <si>
+    <t>Odziv M</t>
+  </si>
+  <si>
+    <t>Preciznost M</t>
+  </si>
+  <si>
+    <t>F1 skor M</t>
+  </si>
+  <si>
+    <t>AUC N</t>
+  </si>
+  <si>
+    <t>Preciznost N</t>
+  </si>
+  <si>
+    <t>AUC M</t>
+  </si>
+  <si>
+    <t>Odziv B</t>
+  </si>
+  <si>
+    <t>Preciznost B</t>
+  </si>
+  <si>
+    <t>F1 skor B</t>
+  </si>
+  <si>
+    <t>AUC B</t>
+  </si>
+  <si>
+    <t> 100%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,13 +151,40 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0F172A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="10">
@@ -243,43 +310,286 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="28">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -298,7 +608,7 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -306,27 +616,6 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -358,7 +647,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -366,8 +655,12 @@
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top/>
-        <bottom/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
         <vertical style="thin">
           <color indexed="64"/>
         </vertical>
@@ -393,7 +686,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -432,7 +725,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -471,7 +764,41 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -485,12 +812,422 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
         <vertical style="thin">
           <color indexed="64"/>
         </vertical>
         <horizontal style="thin">
           <color indexed="64"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -510,27 +1247,7 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -544,157 +1261,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -710,20 +1282,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}" name="Table1" displayName="Table1" ref="A1:I8" totalsRowShown="0" headerRowDxfId="2" dataDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}" name="Table1" displayName="Table1" ref="A1:I8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="26" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
   <autoFilter ref="A1:I8" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{6401034C-4ED1-407E-80E7-E2EB16481849}" name="Metrike" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{06EA2B4A-F014-4F63-905A-7BEAFC1FD8C5}" name="C# 1" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{563E5A62-D0F0-4031-8459-95E4BA9CBDBF}" name="C# 2" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{7D0CB0C7-4969-4EB9-BE3C-DA23CDD44FEF}" name="C# 3" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{1A84A58D-83EA-4727-8B18-4376488C71F5}" name="Prosjek  ± SD" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{1A84A58D-83EA-4727-8B18-4376488C71F5}" name="Prosjek  ± SD" dataDxfId="5">
       <calculatedColumnFormula>FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{6FF159A5-3BC3-4C92-9E1B-3CC1928362A2}" name="Python 1" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{9F166926-181C-4216-B003-78A81AF433F0}" name="Python 2" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{6C1EB1E5-9678-457D-AEA4-1060E1BAE98C}" name="Python 3" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{6FF159A5-3BC3-4C92-9E1B-3CC1928362A2}" name="Python 1" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{9F166926-181C-4216-B003-78A81AF433F0}" name="Python 2" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{6C1EB1E5-9678-457D-AEA4-1060E1BAE98C}" name="Python 3" dataDxfId="2"/>
     <tableColumn id="9" xr3:uid="{11A3B271-D5F8-4C88-8C76-F2361DB67978}" name="Prosjek ± SD2" dataDxfId="1">
+      <calculatedColumnFormula>FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CECF13A1-CDF0-4E28-A11F-4CED5C7B80BB}" name="Table13" displayName="Table13" ref="A1:I13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="27" headerRowBorderDxfId="24" tableBorderDxfId="25" totalsRowBorderDxfId="23">
+  <autoFilter ref="A1:I13" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{7A17A4D7-B4D5-4FCB-A67A-2A0F42F0B6CE}" name="Metrike" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{95EDF1DA-B914-462E-AB64-7BC3F5FA4645}" name="C# 1" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4611FF27-266D-4D37-96AC-D85648DAC03E}" name="C# 2" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{5C582590-5102-47EC-99B8-1973D4C8FEDD}" name="C# 3" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{58433FD4-9BD7-4844-95EE-B57A34492735}" name="Prosjek  ± SD" dataDxfId="18">
+      <calculatedColumnFormula>FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{087F457F-33E5-4759-8129-8C4D449E1FA6}" name="Python 1" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{75421E3E-EB51-4A00-B121-E1A1608AED18}" name="Python 2" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{5D17EC5C-729B-4C98-94ED-711B1588306E}" name="Python 3" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{B6EA0973-CDAB-437D-9237-F730BA0C40C7}" name="Prosjek ± SD2" dataDxfId="14">
       <calculatedColumnFormula>FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1034,7 +1628,7 @@
     <col min="1" max="9" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
@@ -1067,217 +1661,635 @@
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="27">
         <v>184.05</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="27">
         <v>189.8</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="27">
         <v>192.57</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="27" t="str">
         <f t="shared" ref="E2:E8" si="0">FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</f>
         <v>18880,67 ± 434,60</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="27">
         <v>283.79000000000002</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="27">
         <v>330.07</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="27">
         <v>294.75</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="28" t="str">
         <f t="shared" ref="I2:I8" si="1">FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</f>
         <v>30287,00 ± 2418,49</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="5">
         <v>0.8145</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="5">
         <v>0.80730000000000002</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="5">
         <v>0.86909999999999998</v>
       </c>
-      <c r="E3" s="8" t="str">
+      <c r="E3" s="5" t="str">
         <f t="shared" si="0"/>
         <v>83,03 ± 3,38</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="5">
         <v>0.80730000000000002</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="5">
         <v>0.82179999999999997</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="5">
         <v>0.88729999999999998</v>
       </c>
-      <c r="I3" s="9" t="str">
+      <c r="I3" s="29" t="str">
         <f t="shared" si="1"/>
         <v>83,88 ± 4,26</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="8">
-        <v>1</v>
-      </c>
-      <c r="C4" s="8">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8">
-        <v>1</v>
-      </c>
-      <c r="E4" s="8" t="str">
+      <c r="B4" s="5">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5" t="str">
         <f t="shared" si="0"/>
         <v>100,00 ± 0,00</v>
       </c>
-      <c r="F4" s="8">
-        <v>1</v>
-      </c>
-      <c r="G4" s="8">
-        <v>1</v>
-      </c>
-      <c r="H4" s="8">
-        <v>1</v>
-      </c>
-      <c r="I4" s="9" t="str">
+      <c r="F4" s="5">
+        <v>1</v>
+      </c>
+      <c r="G4" s="5">
+        <v>1</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1</v>
+      </c>
+      <c r="I4" s="29" t="str">
         <f t="shared" si="1"/>
         <v>100,00 ± 0,00</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="5">
         <v>0.68810000000000004</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="5">
         <v>0.74760000000000004</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="5">
         <v>0.75060000000000004</v>
       </c>
-      <c r="E5" s="8" t="str">
+      <c r="E5" s="5" t="str">
         <f t="shared" si="0"/>
         <v>72,88 ± 3,53</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="5">
         <v>0.65380000000000005</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="5">
         <v>0.72450000000000003</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="5">
         <v>0.76490000000000002</v>
       </c>
-      <c r="I5" s="9" t="str">
+      <c r="I5" s="29" t="str">
         <f t="shared" si="1"/>
         <v>71,44 ± 5,62</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="5">
         <v>0.69420000000000004</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="5">
         <v>0.7581</v>
       </c>
-      <c r="E6" s="8" t="str">
+      <c r="E6" s="5" t="str">
         <f t="shared" si="0"/>
         <v>72,62 ± 4,52</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="5">
         <v>0.64829999999999999</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="5">
         <v>0.74809999999999999</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="5">
         <v>0.71089999999999998</v>
       </c>
-      <c r="I6" s="9" t="str">
+      <c r="I6" s="29" t="str">
         <f t="shared" si="1"/>
         <v>70,24 ± 5,04</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="5">
         <v>0.68530000000000002</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="5">
         <v>0.75370000000000004</v>
       </c>
-      <c r="E7" s="8" t="str">
+      <c r="E7" s="5" t="str">
         <f t="shared" si="0"/>
         <v>71,95 ± 4,84</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="5">
         <v>0.64939999999999998</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="5">
         <v>0.72089999999999999</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="5">
         <v>0.71479999999999999</v>
       </c>
-      <c r="I7" s="9" t="str">
+      <c r="I7" s="29" t="str">
         <f t="shared" si="1"/>
         <v>69,50 ± 3,96</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="8">
         <v>0.91490000000000005</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="8">
         <v>0.94889999999999997</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="8">
         <v>0.93140000000000001</v>
       </c>
       <c r="E8" s="8" t="str">
         <f t="shared" si="0"/>
         <v>93,17 ± 1,70</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="8">
         <v>0.91459999999999997</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="8">
         <v>0.91869999999999996</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="8">
         <v>0.93210000000000004</v>
       </c>
-      <c r="I8" s="12" t="str">
+      <c r="I8" s="30" t="str">
         <f t="shared" si="1"/>
         <v>92,18 ± 0,92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBF8F9AE-340D-45E7-8E0B-1674AF8EE496}">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="9" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="21">
+        <v>0.4</v>
+      </c>
+      <c r="C2" s="21">
+        <v>0.8</v>
+      </c>
+      <c r="D2" s="22">
+        <v>0.4667</v>
+      </c>
+      <c r="E2" s="13" t="str">
+        <f t="shared" ref="E2:E7" si="0">FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</f>
+        <v>55,56 ± 21,43</v>
+      </c>
+      <c r="F2" s="22">
+        <v>0.23330000000000001</v>
+      </c>
+      <c r="G2" s="23">
+        <v>0.6</v>
+      </c>
+      <c r="H2" s="23">
+        <v>0.2</v>
+      </c>
+      <c r="I2" s="24" t="str">
+        <f t="shared" ref="I2:I13" si="1">FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</f>
+        <v>34,44 ± 22,20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="22">
+        <v>0.26669999999999999</v>
+      </c>
+      <c r="C3" s="22">
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="D3" s="22">
+        <v>0.4118</v>
+      </c>
+      <c r="E3" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>33,88 ± 7,26</v>
+      </c>
+      <c r="F3" s="22">
+        <v>0.2414</v>
+      </c>
+      <c r="G3" s="22">
+        <v>0.35289999999999999</v>
+      </c>
+      <c r="H3" s="21">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>36,48 ± 12,97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="21">
+        <v>0.32</v>
+      </c>
+      <c r="C4" s="22">
+        <v>0.47520000000000001</v>
+      </c>
+      <c r="D4" s="22">
+        <v>0.4375</v>
+      </c>
+      <c r="E4" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>41,09 ± 8,09</v>
+      </c>
+      <c r="F4" s="22">
+        <v>0.23730000000000001</v>
+      </c>
+      <c r="G4" s="25">
+        <v>0.44440000000000002</v>
+      </c>
+      <c r="H4" s="22">
+        <v>0.28570000000000001</v>
+      </c>
+      <c r="I4" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>32,25 ± 10,83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="21">
+        <v>1</v>
+      </c>
+      <c r="C5" s="21">
+        <v>1</v>
+      </c>
+      <c r="D5" s="23">
+        <v>1</v>
+      </c>
+      <c r="E5" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+      <c r="F5" s="23">
+        <v>1</v>
+      </c>
+      <c r="G5" s="21">
+        <v>1</v>
+      </c>
+      <c r="H5" s="21">
+        <v>1</v>
+      </c>
+      <c r="I5" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="21">
+        <v>1</v>
+      </c>
+      <c r="C6" s="21">
+        <v>1</v>
+      </c>
+      <c r="D6" s="23">
+        <v>1</v>
+      </c>
+      <c r="E6" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+      <c r="F6" s="22">
+        <v>0.91559999999999997</v>
+      </c>
+      <c r="G6" s="22">
+        <v>0.97240000000000004</v>
+      </c>
+      <c r="H6" s="22">
+        <v>0.99299999999999999</v>
+      </c>
+      <c r="I6" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>96,03 ± 4,01</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="21">
+        <v>1</v>
+      </c>
+      <c r="C7" s="21">
+        <v>1</v>
+      </c>
+      <c r="D7" s="23">
+        <v>1</v>
+      </c>
+      <c r="E7" s="13" t="str">
+        <f t="shared" si="0"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+      <c r="F7" s="25">
+        <v>0.95589999999999997</v>
+      </c>
+      <c r="G7" s="22">
+        <v>0.98599999999999999</v>
+      </c>
+      <c r="H7" s="22">
+        <v>0.99650000000000005</v>
+      </c>
+      <c r="I7" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>97,95 ± 2,11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="22">
+        <v>0.68269999999999997</v>
+      </c>
+      <c r="C8" s="22">
+        <v>0.54810000000000003</v>
+      </c>
+      <c r="D8" s="22">
+        <v>0.80769999999999997</v>
+      </c>
+      <c r="E8" s="13" t="str">
+        <f t="shared" ref="E8:E12" si="2">FIXED(AVERAGE(B8:D8)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B8:D8)*100, 2, TRUE)</f>
+        <v>67,95 ± 12,98</v>
+      </c>
+      <c r="F8" s="13">
+        <v>0.71150000000000002</v>
+      </c>
+      <c r="G8" s="22">
+        <v>0.64419999999999999</v>
+      </c>
+      <c r="H8" s="22">
+        <v>0.93269999999999997</v>
+      </c>
+      <c r="I8" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>76,28 ± 15,09</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="22">
+        <v>0.79779999999999995</v>
+      </c>
+      <c r="C9" s="22">
+        <v>0.90480000000000005</v>
+      </c>
+      <c r="D9" s="21">
+        <v>0.84</v>
+      </c>
+      <c r="E9" s="13" t="str">
+        <f t="shared" si="2"/>
+        <v>84,75 ± 5,39</v>
+      </c>
+      <c r="F9" s="22">
+        <v>0.80430000000000001</v>
+      </c>
+      <c r="G9" s="22">
+        <v>0.84809999999999997</v>
+      </c>
+      <c r="H9" s="22">
+        <v>0.80169999999999997</v>
+      </c>
+      <c r="I9" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>81,80 ± 2,61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="22">
+        <v>0.73580000000000001</v>
+      </c>
+      <c r="C10" s="25">
+        <v>0.68259999999999998</v>
+      </c>
+      <c r="D10" s="22">
+        <v>0.82350000000000001</v>
+      </c>
+      <c r="E10" s="13" t="str">
+        <f t="shared" si="2"/>
+        <v>74,73 ± 7,12</v>
+      </c>
+      <c r="F10" s="22">
+        <v>0.75509999999999999</v>
+      </c>
+      <c r="G10" s="22">
+        <v>0.73219999999999996</v>
+      </c>
+      <c r="H10" s="22">
+        <v>0.86219999999999997</v>
+      </c>
+      <c r="I10" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>78,32 ± 6,94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="15">
+        <v>0.81799999999999995</v>
+      </c>
+      <c r="C11" s="15">
+        <v>0.89119999999999999</v>
+      </c>
+      <c r="D11" s="15">
+        <v>0.86140000000000005</v>
+      </c>
+      <c r="E11" s="13" t="str">
+        <f t="shared" si="2"/>
+        <v>85,69 ± 3,68</v>
+      </c>
+      <c r="F11" s="15">
+        <v>0.80120000000000002</v>
+      </c>
+      <c r="G11" s="15">
+        <v>0.8196</v>
+      </c>
+      <c r="H11" s="15">
+        <v>0.85019999999999996</v>
+      </c>
+      <c r="I11" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>82,37 ± 2,48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="16">
+        <v>1</v>
+      </c>
+      <c r="C12" s="16">
+        <v>1</v>
+      </c>
+      <c r="D12" s="16">
+        <v>1</v>
+      </c>
+      <c r="E12" s="13" t="str">
+        <f t="shared" si="2"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+      <c r="F12" s="16">
+        <v>1</v>
+      </c>
+      <c r="G12" s="16">
+        <v>1</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>100,00 ± 0,00</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="19">
+        <v>0.92669999999999997</v>
+      </c>
+      <c r="C13" s="19">
+        <v>0.95550000000000002</v>
+      </c>
+      <c r="D13" s="19">
+        <v>0.94320000000000004</v>
+      </c>
+      <c r="E13" s="20" t="str">
+        <f>FIXED(AVERAGE(B13:D13)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B13:D13)*100, 2, TRUE)</f>
+        <v>94,18 ± 1,45</v>
+      </c>
+      <c r="F13" s="19">
+        <v>0.9425</v>
+      </c>
+      <c r="G13" s="19">
+        <v>0.93659999999999999</v>
+      </c>
+      <c r="H13" s="19">
+        <v>0.94620000000000004</v>
+      </c>
+      <c r="I13" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>94,18 ± 0,48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added validation and triaining graphs to doc, fixed image saving in c#.
</commit_message>
<xml_diff>
--- a/Word/rezultati.xlsx
+++ b/Word/rezultati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\source\repos\omarkurtovic\ml-dotnet-vs-python\Word\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F875A91-59F2-4F3D-9848-26D8574E0742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA3A3B4-58DE-48FC-A47F-4B2737282BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5355" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4EAF71C1-AA1B-4CDB-9B0B-819C93A82BA1}"/>
+    <workbookView xWindow="-28920" yWindow="5355" windowWidth="29040" windowHeight="15720" xr2:uid="{4EAF71C1-AA1B-4CDB-9B0B-819C93A82BA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>C# 1</t>
   </si>
@@ -73,13 +73,7 @@
     <t>Makro odziv</t>
   </si>
   <si>
-    <t>78,27%</t>
-  </si>
-  <si>
     <t>Makro F1</t>
-  </si>
-  <si>
-    <t>71,93%</t>
   </si>
   <si>
     <t>Makro AUC</t>
@@ -410,6 +404,40 @@
     <dxf>
       <font>
         <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -420,9 +448,375 @@
         <vertAlign val="baseline"/>
         <sz val="12"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -792,429 +1186,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1250,6 +1221,13 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1261,12 +1239,28 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1282,20 +1276,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}" name="Table1" displayName="Table1" ref="A1:I8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="26" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}" name="Table1" displayName="Table1" ref="A1:I8" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:I8" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{6401034C-4ED1-407E-80E7-E2EB16481849}" name="Metrike" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{06EA2B4A-F014-4F63-905A-7BEAFC1FD8C5}" name="C# 1" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{563E5A62-D0F0-4031-8459-95E4BA9CBDBF}" name="C# 2" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{7D0CB0C7-4969-4EB9-BE3C-DA23CDD44FEF}" name="C# 3" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{1A84A58D-83EA-4727-8B18-4376488C71F5}" name="Prosjek  ± SD" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{6401034C-4ED1-407E-80E7-E2EB16481849}" name="Metrike" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{06EA2B4A-F014-4F63-905A-7BEAFC1FD8C5}" name="C# 1" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{563E5A62-D0F0-4031-8459-95E4BA9CBDBF}" name="C# 2" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{7D0CB0C7-4969-4EB9-BE3C-DA23CDD44FEF}" name="C# 3" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{1A84A58D-83EA-4727-8B18-4376488C71F5}" name="Prosjek  ± SD" dataDxfId="18">
       <calculatedColumnFormula>FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{6FF159A5-3BC3-4C92-9E1B-3CC1928362A2}" name="Python 1" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{9F166926-181C-4216-B003-78A81AF433F0}" name="Python 2" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{6C1EB1E5-9678-457D-AEA4-1060E1BAE98C}" name="Python 3" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{11A3B271-D5F8-4C88-8C76-F2361DB67978}" name="Prosjek ± SD2" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{6FF159A5-3BC3-4C92-9E1B-3CC1928362A2}" name="Python 1" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{9F166926-181C-4216-B003-78A81AF433F0}" name="Python 2" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{6C1EB1E5-9678-457D-AEA4-1060E1BAE98C}" name="Python 3" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{11A3B271-D5F8-4C88-8C76-F2361DB67978}" name="Prosjek ± SD2" dataDxfId="14">
       <calculatedColumnFormula>FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1304,20 +1298,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CECF13A1-CDF0-4E28-A11F-4CED5C7B80BB}" name="Table13" displayName="Table13" ref="A1:I13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="27" headerRowBorderDxfId="24" tableBorderDxfId="25" totalsRowBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CECF13A1-CDF0-4E28-A11F-4CED5C7B80BB}" name="Table13" displayName="Table13" ref="A1:I13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:I13" xr:uid="{BF6174EA-41C6-4A70-8404-3C53704F5F52}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7A17A4D7-B4D5-4FCB-A67A-2A0F42F0B6CE}" name="Metrike" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{95EDF1DA-B914-462E-AB64-7BC3F5FA4645}" name="C# 1" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{4611FF27-266D-4D37-96AC-D85648DAC03E}" name="C# 2" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{5C582590-5102-47EC-99B8-1973D4C8FEDD}" name="C# 3" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{58433FD4-9BD7-4844-95EE-B57A34492735}" name="Prosjek  ± SD" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{7A17A4D7-B4D5-4FCB-A67A-2A0F42F0B6CE}" name="Metrike" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{95EDF1DA-B914-462E-AB64-7BC3F5FA4645}" name="C# 1" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{4611FF27-266D-4D37-96AC-D85648DAC03E}" name="C# 2" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{5C582590-5102-47EC-99B8-1973D4C8FEDD}" name="C# 3" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{58433FD4-9BD7-4844-95EE-B57A34492735}" name="Prosjek  ± SD" dataDxfId="4">
       <calculatedColumnFormula>FIXED(AVERAGE(B2:D2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(B2:D2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{087F457F-33E5-4759-8129-8C4D449E1FA6}" name="Python 1" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{75421E3E-EB51-4A00-B121-E1A1608AED18}" name="Python 2" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{5D17EC5C-729B-4C98-94ED-711B1588306E}" name="Python 3" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{B6EA0973-CDAB-437D-9237-F730BA0C40C7}" name="Prosjek ± SD2" dataDxfId="14">
+    <tableColumn id="6" xr3:uid="{087F457F-33E5-4759-8129-8C4D449E1FA6}" name="Python 1" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{75421E3E-EB51-4A00-B121-E1A1608AED18}" name="Python 2" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{5D17EC5C-729B-4C98-94ED-711B1588306E}" name="Python 3" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{B6EA0973-CDAB-437D-9237-F730BA0C40C7}" name="Prosjek ± SD2" dataDxfId="0">
       <calculatedColumnFormula>FIXED(AVERAGE(F2:H2)*100, 2, TRUE) &amp; " ± " &amp; FIXED(_xlfn.STDEV.S(F2:H2)*100, 2, TRUE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1630,7 +1624,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1642,7 +1636,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>3</v>
@@ -1654,7 +1648,7 @@
         <v>5</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1788,15 +1782,15 @@
       <c r="B6" s="5">
         <v>0.69420000000000004</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>11</v>
+      <c r="C6" s="5">
+        <v>0.78269999999999995</v>
       </c>
       <c r="D6" s="5">
         <v>0.7581</v>
       </c>
       <c r="E6" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>72,62 ± 4,52</v>
+        <v>74,50 ± 4,57</v>
       </c>
       <c r="F6" s="5">
         <v>0.64829999999999999</v>
@@ -1814,20 +1808,20 @@
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="5">
         <v>0.68530000000000002</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>13</v>
+      <c r="C7" s="5">
+        <v>0.71930000000000005</v>
       </c>
       <c r="D7" s="5">
         <v>0.75370000000000004</v>
       </c>
       <c r="E7" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>71,95 ± 4,84</v>
+        <v>71,94 ± 3,42</v>
       </c>
       <c r="F7" s="5">
         <v>0.64939999999999998</v>
@@ -1845,7 +1839,7 @@
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8" s="8">
         <v>0.91490000000000005</v>
@@ -1893,7 +1887,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>0</v>
@@ -1905,7 +1899,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>3</v>
@@ -1917,12 +1911,12 @@
         <v>5</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B2" s="21">
         <v>0.4</v>
@@ -1953,7 +1947,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B3" s="22">
         <v>0.26669999999999999</v>
@@ -1984,7 +1978,7 @@
     </row>
     <row r="4" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="21">
         <v>0.32</v>
@@ -2015,7 +2009,7 @@
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" s="21">
         <v>1</v>
@@ -2046,7 +2040,7 @@
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" s="21">
         <v>1</v>
@@ -2077,7 +2071,7 @@
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B7" s="21">
         <v>1</v>
@@ -2108,7 +2102,7 @@
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="22">
         <v>0.68269999999999997</v>
@@ -2139,7 +2133,7 @@
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="22">
         <v>0.79779999999999995</v>
@@ -2170,7 +2164,7 @@
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" s="22">
         <v>0.73580000000000001</v>
@@ -2201,7 +2195,7 @@
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" s="15">
         <v>0.81799999999999995</v>
@@ -2232,7 +2226,7 @@
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="16">
         <v>1</v>
@@ -2254,7 +2248,7 @@
         <v>1</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I12" s="24" t="str">
         <f t="shared" si="1"/>
@@ -2263,7 +2257,7 @@
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" s="19">
         <v>0.92669999999999997</v>

</xml_diff>